<commit_message>
feat(strategy): add iPhone products and prioritize iPhone in comments and reviews
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="390" yWindow="615" windowWidth="13095" windowHeight="7620" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Affiliate Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affiliate Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1503,6 +1503,146 @@
       <c r="F26" t="inlineStr">
         <is>
           <t>ทิชชู่เปียกสำหรับสัตว์เลี้ยง EGG Pet Wipes 80 แผ่น อ่อนโยน ปลอดภัย</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8AWCoHKL6C</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max ชิป A20 Pro กล้องซูมคมชัด ดีไซน์พรีเมียม สั่งซื้อผ่าน Apple Flagship Store ของแท้ 100% พร้อมรับสิทธิ์ผ่อน 0% SpayLater</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztn-msxxsasoiscl48</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Apple iPhone 17 Pro (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5AsbEphgh5</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Apple iPhone 17 Pro ชิป A19 Pro หน้าจอ ProMotion 120Hz แบตเตอรี่อึดยิ่งขึ้น ระบบกล้องโปร เครื่องศูนย์แท้พร้อมประกันศูนย์ไทย 1 ปีเต็ม</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztf-msuyb0tv79qff4</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>12</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Apple iPhone 16 Plus (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/LnLTzHQeV</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Apple iPhone 16 Plus จอใหญ่เต็มตา แบตเตอรี่อึดทนทาน รองรับ Apple Intelligence เต็มรูปแบบ ชิป A18 เครื่องศูนย์ไทยแท้ ผ่อน 0% ได้</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztg-msuy0uk4gkjo7b</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Apple iPhone 15 (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8fSTPKxXrZ</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Apple iPhone 15 พอร์ต USB-C กล้องหลัก 48MP หน้าจอ Dynamic Island สุดคุ้มค่า ใช้งานลื่นไหลยาวนาน เครื่องศูนย์ไทยแท้</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://store.storeimages.cdn-apple.com/8756/as-images.apple.com/is/iphone-15-finish-select-202309-6-1inch-black?wid=5120&amp;hei=2880&amp;fmt=p-jpg&amp;qlt=80&amp;.v=1692923777972</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(inventory): import 100 trending Shopee affiliate products into curated categories
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1643,6 +1643,246 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>https://store.storeimages.cdn-apple.com/8756/as-images.apple.com/is/iphone-15-finish-select-202309-6-1inch-black?wid=5120&amp;hei=2880&amp;fmt=p-jpg&amp;qlt=80&amp;.v=1692923777972</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>14</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Lifinity ชั้นวางจาน ที่คว่ำจาน 120/105ซม ชั้นวางของในครัว</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1qc9ZkOEib</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Lifinity ชั้นวางจาน ที่คว่ำจาน 120/105ซม ชั้นวางของในครัว ราคา 678.00 บาท</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m6m8v000vb5b5e.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>15</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ANCHI จักรยานพับได้ จักรยานแม่บ้าน จักรยาน แม่บ้าน ญี่ปุ่น เกียร์ 7 ระดับ ตะกร้าเหล็ก จักรยานผู้ใหญ</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4B04MAcB1P</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ANCHI จักรยานพับได้ จักรยานแม่บ้าน จักรยาน แม่บ้าน ญี่ปุ่น เกียร์ 7 ระดับ ตะกร้าเหล็ก จักรยานผู้ใหญ ราคา 1955.00 บาท</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mlw25x1168zm9d.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>เครื่องตัดกิ่งไม้ไร้สาย ตัดแต่งพุ่มไม้ แต่งกิ่งไม้ เครื่องตัดหญ้าไฟฟ้า เลื่อยตัดแต่งสวน ตัดแต่งพุ่มหญ้า</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9KiAVfeVSA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>เครื่องตัดกิ่งไม้ไร้สาย ตัดแต่งพุ่มไม้ แต่งกิ่งไม้ เครื่องตัดหญ้าไฟฟ้า เลื่อยตัดแต่งสวน ตัดแต่งพุ่มหญ้า ราคา 875.00 บาท</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul9-ljuyqy4onhnq0b.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>17</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>【รับประกัน 5ปี】elago เครื่องตัดหญ้าไฟฟ้าไร้สาย แบบพกพา ปรับได้ ยืดหด 5000mAh*2 อุปกรณ์ครบชุด พร้อมแบตเตอรีลิเธียมแท้</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5VVRwdnTF3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>【รับประกัน 5ปี】elago เครื่องตัดหญ้าไฟฟ้าไร้สาย แบบพกพา ปรับได้ ยืดหด 5000mAh*2 อุปกรณ์ครบชุด พร้อมแบตเตอรีลิเธียมแท้ ราคา 634.00 บาท</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mq1py5gj48ox05.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>18</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>[Best Seller] TCL แอร์ Full DC SaveIn AI Inverter ประหยัดไฟ ขนาด 9,200- 24,200 BTU รุ่น TAC-XALCH2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9zxrIvShk4</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>[Best Seller] TCL แอร์ Full DC SaveIn AI Inverter ประหยัดไฟ ขนาด 9,200- 24,200 BTU รุ่น TAC-XALCH2 ราคา 14290.00 บาท</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-msjawf9q8e808c.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>19</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2024 สไตล ์ ใหม ่ Star alpinestars a รถจักรยานยนต ์ Warm Shock-resistant Cycling Jersey Casual แจ ็ คเก ็ ตผู ้ ชายผู ้ หญิงฤดูใบไม ้ ผลิฤดูใบไม ้ ร ่ วงฤดูหนาว Soft Shell แจ ็ คเก ็ ตกันน ้ ํา Star แจ ็ คเก ็ ตสองสี</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3VkNZ0QFA2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2024 สไตล ์ ใหม ่ Star alpinestars a รถจักรยานยนต ์ Warm Shock-resistant Cycling Jersey Casual แจ ็ คเก ็ ตผู ้ ชายผู ้ หญิงฤดูใบไม ้ ผลิฤดูใบไม ้ ร ่ วงฤดูหนาว Soft Shell แจ ็ คเก ็ ตกันน ้ ํา Star แจ ็ คเก ็ ตสองสี ราคา 2107.00 บาท</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-7r98o-luf6vg0dv0xw51.webp</t>
         </is>
       </c>
     </row>

</xml_diff>